<commit_message>
failure reason logging bug fixed
</commit_message>
<xml_diff>
--- a/src/main/resources/rules/rules_dynamic.xlsx
+++ b/src/main/resources/rules/rules_dynamic.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="136">
   <si>
     <t>RuleSet</t>
   </si>
@@ -148,12 +148,105 @@
     <t>getString("/account/validPriDP") == "$1"</t>
   </si>
   <si>
-    <t>set("/account/output/permission", "$param");</t>
+    <t>set("/account/output/evaluationStatus", "$param");</t>
   </si>
   <si>
     <t>set("/account/output/statusTo", "$param");</t>
   </si>
   <si>
+    <t>/account/statusFrom</t>
+  </si>
+  <si>
+    <t>/account/statusTo</t>
+  </si>
+  <si>
+    <t>/account/equityOpenPosition</t>
+  </si>
+  <si>
+    <t>/account/derivativeOpenPosition</t>
+  </si>
+  <si>
+    <t>/account/mtfOpenPosn</t>
+  </si>
+  <si>
+    <t>/account/marginPledge</t>
+  </si>
+  <si>
+    <t>/account/cuspa</t>
+  </si>
+  <si>
+    <t>/account/noOFSActivityLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noBuybackActivityLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noOpenOfferActivityLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noIPOSubscriptionLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noSGBTransactionLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noMutualFundTransactionLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noInsuranceTransactionLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noNCDBondActivityLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noNSDLOrCDSLActivityLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noApprovedPayInPayOutLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noKRAInitialOrModificationLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noCKYCUploadOrModificationLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noApprovedCRFLast24Months</t>
+  </si>
+  <si>
+    <t>/account/noExchangeTradingLast24Months</t>
+  </si>
+  <si>
+    <t>/account/notTradedOnCurrentDate</t>
+  </si>
+  <si>
+    <t>/account/activeNACH</t>
+  </si>
+  <si>
+    <t>/account/activeSIP</t>
+  </si>
+  <si>
+    <t>/account/valid3KYC/adhaar</t>
+  </si>
+  <si>
+    <t>/account/valid3KYC/pan</t>
+  </si>
+  <si>
+    <t>/account/valid3KYC/passport</t>
+  </si>
+  <si>
+    <t>/account/compiledKRA</t>
+  </si>
+  <si>
+    <t>/account/validCKYCNum</t>
+  </si>
+  <si>
+    <t>/account/validPriBankAcc</t>
+  </si>
+  <si>
+    <t>/account/validPriDP</t>
+  </si>
+  <si>
     <t>Initial Status</t>
   </si>
   <si>
@@ -320,6 +413,12 @@
   </si>
   <si>
     <t>SELLING ONLY</t>
+  </si>
+  <si>
+    <t>activeToSelllingOnly2</t>
+  </si>
+  <si>
+    <t>activeToSelllingOnly3</t>
   </si>
 </sst>
 </file>
@@ -357,7 +456,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -432,6 +531,12 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="18"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -499,7 +604,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -545,13 +650,16 @@
     <xf numFmtId="49" fontId="0" fillId="9" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="10" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="10" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -582,6 +690,7 @@
       <rgbColor rgb="fff19d64"/>
       <rgbColor rgb="ff93c175"/>
       <rgbColor rgb="ffaaaaaa"/>
+      <rgbColor rgb="fff19d64"/>
       <rgbColor rgb="ffadcdea"/>
     </indexedColors>
   </colors>
@@ -1617,7 +1726,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AI18"/>
+  <dimension ref="A1:AI19"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="2" width="28.6719" style="1" customWidth="1"/>
@@ -2088,861 +2197,1100 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" ht="18.95" customHeight="1">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+    <row r="9" ht="12.9" customHeight="1">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
       <c r="C9" t="s" s="15">
         <v>47</v>
       </c>
-      <c r="D9" t="s" s="16">
+      <c r="D9" t="s" s="15">
         <v>48</v>
       </c>
-      <c r="E9" t="s" s="16">
+      <c r="E9" t="s" s="15">
         <v>49</v>
       </c>
-      <c r="F9" t="s" s="16">
+      <c r="F9" t="s" s="15">
         <v>50</v>
       </c>
-      <c r="G9" t="s" s="16">
+      <c r="G9" t="s" s="15">
         <v>51</v>
       </c>
-      <c r="H9" t="s" s="16">
+      <c r="H9" t="s" s="15">
         <v>52</v>
       </c>
-      <c r="I9" t="s" s="16">
+      <c r="I9" t="s" s="15">
         <v>53</v>
       </c>
-      <c r="J9" t="s" s="16">
+      <c r="J9" t="s" s="15">
         <v>54</v>
       </c>
-      <c r="K9" t="s" s="16">
+      <c r="K9" t="s" s="11">
         <v>55</v>
       </c>
-      <c r="L9" t="s" s="16">
+      <c r="L9" t="s" s="11">
         <v>56</v>
       </c>
-      <c r="M9" t="s" s="16">
+      <c r="M9" t="s" s="11">
         <v>57</v>
       </c>
-      <c r="N9" t="s" s="16">
+      <c r="N9" t="s" s="11">
         <v>58</v>
       </c>
-      <c r="O9" t="s" s="16">
+      <c r="O9" t="s" s="11">
         <v>59</v>
       </c>
-      <c r="P9" t="s" s="16">
+      <c r="P9" t="s" s="11">
         <v>60</v>
       </c>
-      <c r="Q9" t="s" s="16">
+      <c r="Q9" t="s" s="11">
         <v>61</v>
       </c>
-      <c r="R9" t="s" s="16">
+      <c r="R9" t="s" s="11">
         <v>62</v>
       </c>
-      <c r="S9" t="s" s="16">
+      <c r="S9" t="s" s="11">
         <v>63</v>
       </c>
-      <c r="T9" t="s" s="16">
+      <c r="T9" t="s" s="11">
         <v>64</v>
       </c>
-      <c r="U9" t="s" s="16">
+      <c r="U9" t="s" s="11">
         <v>65</v>
       </c>
-      <c r="V9" t="s" s="16">
+      <c r="V9" t="s" s="11">
         <v>66</v>
       </c>
-      <c r="W9" t="s" s="16">
+      <c r="W9" t="s" s="11">
         <v>67</v>
       </c>
-      <c r="X9" t="s" s="16">
+      <c r="X9" t="s" s="11">
         <v>68</v>
       </c>
-      <c r="Y9" t="s" s="16">
+      <c r="Y9" t="s" s="11">
         <v>69</v>
       </c>
-      <c r="Z9" t="s" s="16">
+      <c r="Z9" t="s" s="11">
         <v>70</v>
       </c>
-      <c r="AA9" t="s" s="16">
+      <c r="AA9" t="s" s="11">
         <v>71</v>
       </c>
-      <c r="AB9" t="s" s="16">
+      <c r="AB9" t="s" s="11">
         <v>72</v>
       </c>
-      <c r="AC9" t="s" s="16">
+      <c r="AC9" t="s" s="11">
         <v>73</v>
       </c>
-      <c r="AD9" t="s" s="16">
+      <c r="AD9" t="s" s="11">
         <v>74</v>
       </c>
-      <c r="AE9" t="s" s="16">
+      <c r="AE9" t="s" s="11">
         <v>75</v>
       </c>
-      <c r="AF9" t="s" s="16">
+      <c r="AF9" t="s" s="11">
         <v>76</v>
       </c>
-      <c r="AG9" t="s" s="16">
+      <c r="AG9" t="s" s="11">
         <v>77</v>
       </c>
-      <c r="AH9" t="s" s="16">
+      <c r="AH9" s="14"/>
+      <c r="AI9" s="14"/>
+    </row>
+    <row r="10" ht="18.95" customHeight="1">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
+      <c r="C10" t="s" s="16">
         <v>78</v>
       </c>
-      <c r="AI9" t="s" s="17">
+      <c r="D10" t="s" s="17">
         <v>79</v>
       </c>
-    </row>
-    <row r="10" ht="12.9" customHeight="1">
-      <c r="A10" t="s" s="2">
+      <c r="E10" t="s" s="17">
         <v>80</v>
       </c>
-      <c r="B10" t="s" s="2">
+      <c r="F10" t="s" s="17">
         <v>81</v>
       </c>
-      <c r="C10" t="s" s="18">
+      <c r="G10" t="s" s="17">
         <v>82</v>
       </c>
-      <c r="D10" t="s" s="18">
+      <c r="H10" t="s" s="17">
         <v>83</v>
       </c>
-      <c r="E10" t="s" s="18">
+      <c r="I10" t="s" s="17">
         <v>84</v>
       </c>
-      <c r="F10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="G10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="H10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="I10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="J10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="K10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="L10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="M10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="N10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="O10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="P10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Q10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="R10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="S10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="T10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="U10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="V10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="W10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="X10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Y10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Z10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AA10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AB10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AC10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AD10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AE10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AF10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AG10" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AH10" t="s" s="18">
+      <c r="J10" t="s" s="17">
         <v>85</v>
       </c>
+      <c r="K10" t="s" s="17">
+        <v>86</v>
+      </c>
+      <c r="L10" t="s" s="17">
+        <v>87</v>
+      </c>
+      <c r="M10" t="s" s="17">
+        <v>88</v>
+      </c>
+      <c r="N10" t="s" s="17">
+        <v>89</v>
+      </c>
+      <c r="O10" t="s" s="17">
+        <v>90</v>
+      </c>
+      <c r="P10" t="s" s="17">
+        <v>91</v>
+      </c>
+      <c r="Q10" t="s" s="17">
+        <v>92</v>
+      </c>
+      <c r="R10" t="s" s="17">
+        <v>93</v>
+      </c>
+      <c r="S10" t="s" s="17">
+        <v>94</v>
+      </c>
+      <c r="T10" t="s" s="17">
+        <v>95</v>
+      </c>
+      <c r="U10" t="s" s="17">
+        <v>96</v>
+      </c>
+      <c r="V10" t="s" s="17">
+        <v>97</v>
+      </c>
+      <c r="W10" t="s" s="17">
+        <v>98</v>
+      </c>
+      <c r="X10" t="s" s="17">
+        <v>99</v>
+      </c>
+      <c r="Y10" t="s" s="17">
+        <v>100</v>
+      </c>
+      <c r="Z10" t="s" s="17">
+        <v>101</v>
+      </c>
+      <c r="AA10" t="s" s="17">
+        <v>102</v>
+      </c>
+      <c r="AB10" t="s" s="17">
+        <v>103</v>
+      </c>
+      <c r="AC10" t="s" s="17">
+        <v>104</v>
+      </c>
+      <c r="AD10" t="s" s="17">
+        <v>105</v>
+      </c>
+      <c r="AE10" t="s" s="17">
+        <v>106</v>
+      </c>
+      <c r="AF10" t="s" s="17">
+        <v>107</v>
+      </c>
+      <c r="AG10" t="s" s="17">
+        <v>108</v>
+      </c>
+      <c r="AH10" t="s" s="17">
+        <v>109</v>
+      </c>
       <c r="AI10" t="s" s="18">
-        <v>86</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" ht="12.9" customHeight="1">
       <c r="A11" t="s" s="2">
-        <v>87</v>
+        <v>111</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="C11" t="s" s="18">
-        <v>82</v>
-      </c>
-      <c r="D11" t="s" s="18">
-        <v>83</v>
-      </c>
-      <c r="E11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="F11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="G11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="H11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="I11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="J11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="K11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="L11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="M11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="N11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="O11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="P11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Q11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="R11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="S11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="T11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="U11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="V11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="W11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="X11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Y11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Z11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AA11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AB11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AC11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AD11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AE11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AF11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AG11" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AH11" t="s" s="18">
-        <v>85</v>
-      </c>
-      <c r="AI11" t="s" s="18">
-        <v>86</v>
+        <v>112</v>
+      </c>
+      <c r="C11" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D11" t="s" s="19">
+        <v>114</v>
+      </c>
+      <c r="E11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AG11" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AH11" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI11" t="s" s="19">
+        <v>117</v>
       </c>
     </row>
     <row r="12" ht="12.9" customHeight="1">
       <c r="A12" t="s" s="2">
-        <v>88</v>
+        <v>118</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>89</v>
-      </c>
-      <c r="C12" t="s" s="18">
-        <v>82</v>
-      </c>
-      <c r="D12" t="s" s="18">
-        <v>90</v>
-      </c>
-      <c r="E12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="F12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="G12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="H12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="I12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="J12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="K12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="L12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="M12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="N12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="O12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="P12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Q12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="R12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="S12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="T12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="U12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="V12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="W12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="X12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Y12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Z12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AA12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AB12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AC12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AD12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AE12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AF12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AG12" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AH12" t="s" s="18">
-        <v>85</v>
-      </c>
-      <c r="AI12" t="s" s="18">
-        <v>91</v>
+        <v>112</v>
+      </c>
+      <c r="C12" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D12" t="s" s="19">
+        <v>114</v>
+      </c>
+      <c r="E12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AG12" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AH12" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI12" t="s" s="19">
+        <v>117</v>
       </c>
     </row>
     <row r="13" ht="12.9" customHeight="1">
       <c r="A13" t="s" s="2">
-        <v>92</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="C13" t="s" s="18">
-        <v>82</v>
-      </c>
-      <c r="D13" t="s" s="18">
-        <v>94</v>
-      </c>
-      <c r="E13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="F13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="G13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="H13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="I13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="J13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="K13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="L13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="M13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="N13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="O13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="P13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Q13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="R13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="S13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="T13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="U13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="V13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="W13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="X13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Y13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Z13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AA13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AB13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AC13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AD13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AE13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AF13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AG13" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AH13" t="s" s="18">
-        <v>85</v>
-      </c>
-      <c r="AI13" t="s" s="18">
-        <v>95</v>
+        <v>120</v>
+      </c>
+      <c r="C13" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D13" t="s" s="19">
+        <v>121</v>
+      </c>
+      <c r="E13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AG13" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AH13" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI13" t="s" s="19">
+        <v>122</v>
       </c>
     </row>
     <row r="14" ht="12.9" customHeight="1">
       <c r="A14" t="s" s="2">
-        <v>96</v>
+        <v>123</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>97</v>
-      </c>
-      <c r="C14" t="s" s="18">
-        <v>90</v>
-      </c>
-      <c r="D14" t="s" s="18">
-        <v>83</v>
-      </c>
-      <c r="E14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="F14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="G14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="H14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="I14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="J14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="K14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="L14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="M14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="N14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="O14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="P14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Q14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="R14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="S14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="T14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="U14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="V14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="W14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="X14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Y14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Z14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AA14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AB14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AC14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AD14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AE14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AF14" t="s" s="18">
-        <v>98</v>
-      </c>
-      <c r="AG14" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AH14" t="s" s="18">
-        <v>85</v>
-      </c>
-      <c r="AI14" t="s" s="18">
-        <v>86</v>
+        <v>124</v>
+      </c>
+      <c r="C14" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D14" t="s" s="19">
+        <v>125</v>
+      </c>
+      <c r="E14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AG14" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AH14" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI14" t="s" s="19">
+        <v>126</v>
       </c>
     </row>
     <row r="15" ht="12.9" customHeight="1">
       <c r="A15" t="s" s="2">
-        <v>99</v>
+        <v>127</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>100</v>
-      </c>
-      <c r="C15" t="s" s="18">
-        <v>82</v>
-      </c>
-      <c r="D15" t="s" s="18">
-        <v>101</v>
-      </c>
-      <c r="E15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="F15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="G15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="H15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="I15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="J15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="K15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="L15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="M15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="N15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="O15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="P15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Q15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="R15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="S15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="T15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="U15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="V15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="W15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="X15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Y15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="Z15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AA15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AB15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AC15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AD15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AE15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AF15" t="s" s="18">
-        <v>84</v>
-      </c>
-      <c r="AG15" t="s" s="18">
-        <v>98</v>
-      </c>
-      <c r="AH15" t="s" s="18">
-        <v>85</v>
-      </c>
-      <c r="AI15" t="s" s="18">
-        <v>102</v>
+        <v>128</v>
+      </c>
+      <c r="C15" t="s" s="19">
+        <v>121</v>
+      </c>
+      <c r="D15" t="s" s="19">
+        <v>114</v>
+      </c>
+      <c r="E15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF15" t="s" s="19">
+        <v>129</v>
+      </c>
+      <c r="AG15" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AH15" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI15" t="s" s="19">
+        <v>117</v>
       </c>
     </row>
     <row r="16" ht="12.9" customHeight="1">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="18"/>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="18"/>
-      <c r="I16" s="18"/>
-      <c r="J16" s="18"/>
-      <c r="K16" s="18"/>
-      <c r="L16" s="18"/>
-      <c r="M16" s="18"/>
-      <c r="N16" s="18"/>
-      <c r="O16" s="18"/>
-      <c r="P16" s="18"/>
-      <c r="Q16" s="18"/>
-      <c r="R16" s="18"/>
-      <c r="S16" s="18"/>
-      <c r="T16" s="18"/>
-      <c r="U16" s="18"/>
-      <c r="V16" s="18"/>
-      <c r="W16" s="18"/>
-      <c r="X16" s="18"/>
-      <c r="Y16" s="18"/>
-      <c r="Z16" s="18"/>
-      <c r="AA16" s="18"/>
-      <c r="AB16" s="18"/>
-      <c r="AC16" s="18"/>
-      <c r="AD16" s="18"/>
-      <c r="AE16" s="18"/>
-      <c r="AF16" s="18"/>
-      <c r="AG16" s="18"/>
-      <c r="AH16" s="18"/>
-      <c r="AI16" s="18"/>
+      <c r="A16" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="B16" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="C16" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D16" t="s" s="19">
+        <v>132</v>
+      </c>
+      <c r="E16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF16" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AG16" t="s" s="19">
+        <v>129</v>
+      </c>
+      <c r="AH16" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI16" t="s" s="19">
+        <v>133</v>
+      </c>
     </row>
     <row r="17" ht="12.9" customHeight="1">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="18"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="18"/>
-      <c r="I17" s="18"/>
-      <c r="J17" s="18"/>
-      <c r="K17" s="18"/>
-      <c r="L17" s="18"/>
-      <c r="M17" s="18"/>
-      <c r="N17" s="18"/>
-      <c r="O17" s="18"/>
-      <c r="P17" s="18"/>
-      <c r="Q17" s="18"/>
-      <c r="R17" s="18"/>
-      <c r="S17" s="18"/>
-      <c r="T17" s="18"/>
-      <c r="U17" s="18"/>
-      <c r="V17" s="18"/>
-      <c r="W17" s="18"/>
-      <c r="X17" s="18"/>
-      <c r="Y17" s="18"/>
-      <c r="Z17" s="18"/>
-      <c r="AA17" s="18"/>
-      <c r="AB17" s="18"/>
-      <c r="AC17" s="18"/>
-      <c r="AD17" s="18"/>
-      <c r="AE17" s="18"/>
-      <c r="AF17" s="18"/>
-      <c r="AG17" s="18"/>
-      <c r="AH17" s="18"/>
-      <c r="AI17" s="18"/>
+      <c r="A17" t="s" s="2">
+        <v>134</v>
+      </c>
+      <c r="B17" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="C17" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D17" t="s" s="19">
+        <v>132</v>
+      </c>
+      <c r="E17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AF17" t="s" s="19">
+        <v>129</v>
+      </c>
+      <c r="AG17" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AH17" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI17" t="s" s="19">
+        <v>133</v>
+      </c>
     </row>
     <row r="18" ht="12.9" customHeight="1">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="18"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="18"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="18"/>
-      <c r="K18" s="18"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="18"/>
-      <c r="N18" s="18"/>
-      <c r="O18" s="18"/>
-      <c r="P18" s="18"/>
-      <c r="Q18" s="18"/>
-      <c r="R18" s="18"/>
-      <c r="S18" s="18"/>
-      <c r="T18" s="18"/>
-      <c r="U18" s="18"/>
-      <c r="V18" s="18"/>
-      <c r="W18" s="18"/>
-      <c r="X18" s="18"/>
-      <c r="Y18" s="18"/>
-      <c r="Z18" s="18"/>
-      <c r="AA18" s="18"/>
-      <c r="AB18" s="18"/>
-      <c r="AC18" s="18"/>
-      <c r="AD18" s="18"/>
-      <c r="AE18" s="18"/>
-      <c r="AF18" s="18"/>
-      <c r="AG18" s="18"/>
-      <c r="AH18" s="18"/>
-      <c r="AI18" s="18"/>
+      <c r="A18" t="s" s="2">
+        <v>135</v>
+      </c>
+      <c r="B18" t="s" s="2">
+        <v>131</v>
+      </c>
+      <c r="C18" t="s" s="19">
+        <v>113</v>
+      </c>
+      <c r="D18" t="s" s="19">
+        <v>132</v>
+      </c>
+      <c r="E18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="F18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="G18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="H18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="I18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="J18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="K18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="L18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="M18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="N18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="O18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="P18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Q18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="R18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="S18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="T18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="U18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="V18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="W18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="X18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Y18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="Z18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AA18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AB18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AC18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AD18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AE18" t="s" s="19">
+        <v>129</v>
+      </c>
+      <c r="AF18" t="s" s="19">
+        <v>115</v>
+      </c>
+      <c r="AG18" t="s" s="19">
+        <v>129</v>
+      </c>
+      <c r="AH18" t="s" s="19">
+        <v>116</v>
+      </c>
+      <c r="AI18" t="s" s="19">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="19" ht="12.9" customHeight="1">
+      <c r="A19" s="2"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="19"/>
+      <c r="I19" s="19"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="19"/>
+      <c r="L19" s="19"/>
+      <c r="M19" s="19"/>
+      <c r="N19" s="19"/>
+      <c r="O19" s="19"/>
+      <c r="P19" s="19"/>
+      <c r="Q19" s="19"/>
+      <c r="R19" s="19"/>
+      <c r="S19" s="19"/>
+      <c r="T19" s="19"/>
+      <c r="U19" s="19"/>
+      <c r="V19" s="19"/>
+      <c r="W19" s="19"/>
+      <c r="X19" s="19"/>
+      <c r="Y19" s="19"/>
+      <c r="Z19" s="19"/>
+      <c r="AA19" s="19"/>
+      <c r="AB19" s="19"/>
+      <c r="AC19" s="19"/>
+      <c r="AD19" s="19"/>
+      <c r="AE19" s="19"/>
+      <c r="AF19" s="19"/>
+      <c r="AG19" s="19"/>
+      <c r="AH19" s="19"/>
+      <c r="AI19" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
faiure reason log with added description
</commit_message>
<xml_diff>
--- a/src/main/resources/rules/rules_dynamic.xlsx
+++ b/src/main/resources/rules/rules_dynamic.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="166">
   <si>
     <t>RuleSet</t>
   </si>
@@ -148,7 +148,7 @@
     <t>getString("/account/validPriDP") == "$1"</t>
   </si>
   <si>
-    <t>set("/account/output/evaluationStatus", "$param");</t>
+    <t>set("/account/output/evalResult", "$param");</t>
   </si>
   <si>
     <t>set("/account/output/statusTo", "$param");</t>
@@ -247,6 +247,93 @@
     <t>/account/validPriDP</t>
   </si>
   <si>
+    <t>Equity Open Position must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Derivative Open Position must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>MTF Open Position must $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Margin Pledge condition must be $expected but $actual</t>
+  </si>
+  <si>
+    <t>CUSPA must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>OFS Activity for last 24 months must be $expected but $actual</t>
+  </si>
+  <si>
+    <t>Buy back activity for last 24 months must be $expected by $actual</t>
+  </si>
+  <si>
+    <t>Open offer activity for last 24 months must be $expected but $actual</t>
+  </si>
+  <si>
+    <t>IPO Subscription activity for last 24 month must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>SGB Transaction in last 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Mutual fund transactions for last 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Insurance transaction activity for the past 24 months must be $expected but $actual</t>
+  </si>
+  <si>
+    <t>NCD Bond activity for last 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>NSDL or CDSL activity for last 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Approved pay in Pay out for the past 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>KRAI initialization or modification activity for the past 24 months must be $expected but $actual</t>
+  </si>
+  <si>
+    <t>CKYC upload or modification activity for the past 24 months must be $expected but $actual</t>
+  </si>
+  <si>
+    <t>Approved CRF within last 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Exchange trading activity for the past 24 months must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Traded on current date must be $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Expected active NACH is $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Expected active SIP is $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Expected a valid adhaar, $expected but not found, $actual</t>
+  </si>
+  <si>
+    <t>Expected a valid PAN, $expected but not found, $actual</t>
+  </si>
+  <si>
+    <t>Expected a valid Passport, $expected but not found, $actual</t>
+  </si>
+  <si>
+    <t>Compiled KRA expected $expected, but found $actual</t>
+  </si>
+  <si>
+    <t>Valid CKYC Number expected, $expected, found $actual</t>
+  </si>
+  <si>
+    <t>Expected a valid primary brank account, $expected but found $actual</t>
+  </si>
+  <si>
+    <t>Primary DP must be $expected but found $actual</t>
+  </si>
+  <si>
     <t>Initial Status</t>
   </si>
   <si>
@@ -340,7 +427,7 @@
     <t>Valid Primary DP</t>
   </si>
   <si>
-    <t>Allowed</t>
+    <t>Evaluation Result</t>
   </si>
   <si>
     <t>Status</t>
@@ -358,6 +445,9 @@
     <t>F</t>
   </si>
   <si>
+    <t>Y</t>
+  </si>
+  <si>
     <t>N</t>
   </si>
   <si>
@@ -370,6 +460,9 @@
     <t>activeToFreeze2</t>
   </si>
   <si>
+    <t>activeToFreeze3</t>
+  </si>
+  <si>
     <t>activeToSuspend1</t>
   </si>
   <si>
@@ -398,9 +491,6 @@
   </si>
   <si>
     <t>sellingToFreeze</t>
-  </si>
-  <si>
-    <t>Y</t>
   </si>
   <si>
     <t>activeToSelllingOnly1</t>
@@ -456,7 +546,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -537,6 +627,12 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="19"/>
+        <bgColor auto="1"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -604,7 +700,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -653,13 +749,16 @@
     <xf numFmtId="49" fontId="0" fillId="10" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="11" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="11" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="11" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="12" borderId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="11" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="12" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="12" borderId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -691,6 +790,7 @@
       <rgbColor rgb="ff93c175"/>
       <rgbColor rgb="ffaaaaaa"/>
       <rgbColor rgb="fff19d64"/>
+      <rgbColor rgb="ffb7d6a3"/>
       <rgbColor rgb="ffadcdea"/>
     </indexedColors>
   </colors>
@@ -1726,19 +1826,30 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AI19"/>
+  <dimension ref="A1:AI21"/>
   <sheetFormatPr defaultColWidth="16.3333" defaultRowHeight="15.4" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="2" width="28.6719" style="1" customWidth="1"/>
-    <col min="3" max="10" width="45.6719" style="1" customWidth="1"/>
-    <col min="11" max="11" width="49.9609" style="1" customWidth="1"/>
-    <col min="12" max="12" width="52.0781" style="1" customWidth="1"/>
-    <col min="13" max="14" width="49.2656" style="1" customWidth="1"/>
-    <col min="15" max="15" width="53.6719" style="1" customWidth="1"/>
-    <col min="16" max="16" width="51.8516" style="1" customWidth="1"/>
-    <col min="17" max="17" width="49.2656" style="1" customWidth="1"/>
-    <col min="18" max="18" width="51" style="1" customWidth="1"/>
-    <col min="19" max="33" width="49.2656" style="1" customWidth="1"/>
+    <col min="3" max="5" width="45.6719" style="1" customWidth="1"/>
+    <col min="6" max="6" width="47.6719" style="1" customWidth="1"/>
+    <col min="7" max="9" width="45.6719" style="1" customWidth="1"/>
+    <col min="10" max="10" width="47.3516" style="1" customWidth="1"/>
+    <col min="11" max="11" width="50.1719" style="1" customWidth="1"/>
+    <col min="12" max="12" width="53.3672" style="1" customWidth="1"/>
+    <col min="13" max="13" width="60.5" style="1" customWidth="1"/>
+    <col min="14" max="14" width="54.5" style="1" customWidth="1"/>
+    <col min="15" max="15" width="62" style="1" customWidth="1"/>
+    <col min="16" max="16" width="63.6719" style="1" customWidth="1"/>
+    <col min="17" max="17" width="56.6719" style="1" customWidth="1"/>
+    <col min="18" max="18" width="59" style="1" customWidth="1"/>
+    <col min="19" max="19" width="64.6719" style="1" customWidth="1"/>
+    <col min="20" max="20" width="73.7266" style="1" customWidth="1"/>
+    <col min="21" max="21" width="68.8516" style="1" customWidth="1"/>
+    <col min="22" max="22" width="56.1719" style="1" customWidth="1"/>
+    <col min="23" max="23" width="65.1719" style="1" customWidth="1"/>
+    <col min="24" max="31" width="49.2656" style="1" customWidth="1"/>
+    <col min="32" max="32" width="52.5" style="1" customWidth="1"/>
+    <col min="33" max="33" width="49.2656" style="1" customWidth="1"/>
     <col min="34" max="35" width="40.1719" style="1" customWidth="1"/>
     <col min="36" max="16384" width="16.3516" style="1" customWidth="1"/>
   </cols>
@@ -1866,7 +1977,7 @@
       <c r="AH3" s="4"/>
       <c r="AI3" s="4"/>
     </row>
-    <row r="4" ht="21.05" customHeight="1">
+    <row r="4" ht="19.1" customHeight="1">
       <c r="A4" s="6"/>
       <c r="B4" s="6"/>
       <c r="C4" t="s" s="5">
@@ -1905,7 +2016,7 @@
       <c r="AH4" s="4"/>
       <c r="AI4" s="4"/>
     </row>
-    <row r="5" ht="32.9" customHeight="1">
+    <row r="5" ht="26.45" customHeight="1">
       <c r="A5" s="2"/>
       <c r="B5" s="2"/>
       <c r="C5" t="s" s="3">
@@ -2197,7 +2308,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="9" ht="12.9" customHeight="1">
+    <row r="9" ht="12.9" customHeight="1" hidden="1">
       <c r="A9" s="6"/>
       <c r="B9" s="6"/>
       <c r="C9" t="s" s="15">
@@ -2296,1001 +2407,1203 @@
       <c r="AH9" s="14"/>
       <c r="AI9" s="14"/>
     </row>
-    <row r="10" ht="18.95" customHeight="1">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" t="s" s="16">
+    <row r="10" ht="12.9" customHeight="1" hidden="1">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" t="s" s="16">
         <v>78</v>
       </c>
-      <c r="D10" t="s" s="17">
+      <c r="F10" t="s" s="16">
         <v>79</v>
       </c>
-      <c r="E10" t="s" s="17">
+      <c r="G10" t="s" s="16">
         <v>80</v>
       </c>
-      <c r="F10" t="s" s="17">
+      <c r="H10" t="s" s="16">
         <v>81</v>
       </c>
-      <c r="G10" t="s" s="17">
+      <c r="I10" t="s" s="16">
         <v>82</v>
       </c>
-      <c r="H10" t="s" s="17">
+      <c r="J10" t="s" s="16">
         <v>83</v>
       </c>
-      <c r="I10" t="s" s="17">
+      <c r="K10" t="s" s="16">
         <v>84</v>
       </c>
-      <c r="J10" t="s" s="17">
+      <c r="L10" t="s" s="16">
         <v>85</v>
       </c>
-      <c r="K10" t="s" s="17">
+      <c r="M10" t="s" s="16">
         <v>86</v>
       </c>
-      <c r="L10" t="s" s="17">
+      <c r="N10" t="s" s="16">
         <v>87</v>
       </c>
-      <c r="M10" t="s" s="17">
+      <c r="O10" t="s" s="16">
         <v>88</v>
       </c>
-      <c r="N10" t="s" s="17">
+      <c r="P10" t="s" s="16">
         <v>89</v>
       </c>
-      <c r="O10" t="s" s="17">
+      <c r="Q10" t="s" s="16">
         <v>90</v>
       </c>
-      <c r="P10" t="s" s="17">
+      <c r="R10" t="s" s="16">
         <v>91</v>
       </c>
-      <c r="Q10" t="s" s="17">
+      <c r="S10" t="s" s="16">
         <v>92</v>
       </c>
-      <c r="R10" t="s" s="17">
+      <c r="T10" t="s" s="16">
         <v>93</v>
       </c>
-      <c r="S10" t="s" s="17">
+      <c r="U10" t="s" s="16">
         <v>94</v>
       </c>
-      <c r="T10" t="s" s="17">
+      <c r="V10" t="s" s="16">
         <v>95</v>
       </c>
-      <c r="U10" t="s" s="17">
+      <c r="W10" t="s" s="16">
         <v>96</v>
       </c>
-      <c r="V10" t="s" s="17">
+      <c r="X10" t="s" s="16">
         <v>97</v>
       </c>
-      <c r="W10" t="s" s="17">
+      <c r="Y10" t="s" s="16">
         <v>98</v>
       </c>
-      <c r="X10" t="s" s="17">
+      <c r="Z10" t="s" s="16">
         <v>99</v>
       </c>
-      <c r="Y10" t="s" s="17">
+      <c r="AA10" t="s" s="16">
         <v>100</v>
       </c>
-      <c r="Z10" t="s" s="17">
+      <c r="AB10" t="s" s="16">
         <v>101</v>
       </c>
-      <c r="AA10" t="s" s="17">
+      <c r="AC10" t="s" s="16">
         <v>102</v>
       </c>
-      <c r="AB10" t="s" s="17">
+      <c r="AD10" t="s" s="16">
         <v>103</v>
       </c>
-      <c r="AC10" t="s" s="17">
+      <c r="AE10" t="s" s="16">
         <v>104</v>
       </c>
-      <c r="AD10" t="s" s="17">
+      <c r="AF10" t="s" s="16">
         <v>105</v>
       </c>
-      <c r="AE10" t="s" s="17">
+      <c r="AG10" t="s" s="16">
         <v>106</v>
       </c>
-      <c r="AF10" t="s" s="17">
+      <c r="AH10" s="14"/>
+      <c r="AI10" s="14"/>
+    </row>
+    <row r="11" ht="18.95" customHeight="1">
+      <c r="A11" s="2"/>
+      <c r="B11" s="2"/>
+      <c r="C11" t="s" s="17">
         <v>107</v>
       </c>
-      <c r="AG10" t="s" s="17">
+      <c r="D11" t="s" s="18">
         <v>108</v>
       </c>
-      <c r="AH10" t="s" s="17">
+      <c r="E11" t="s" s="18">
         <v>109</v>
       </c>
-      <c r="AI10" t="s" s="18">
+      <c r="F11" t="s" s="18">
         <v>110</v>
       </c>
-    </row>
-    <row r="11" ht="12.9" customHeight="1">
-      <c r="A11" t="s" s="2">
+      <c r="G11" t="s" s="18">
         <v>111</v>
       </c>
-      <c r="B11" t="s" s="2">
+      <c r="H11" t="s" s="18">
         <v>112</v>
       </c>
-      <c r="C11" t="s" s="19">
+      <c r="I11" t="s" s="18">
         <v>113</v>
       </c>
-      <c r="D11" t="s" s="19">
+      <c r="J11" t="s" s="18">
         <v>114</v>
       </c>
-      <c r="E11" t="s" s="19">
+      <c r="K11" t="s" s="18">
         <v>115</v>
       </c>
-      <c r="F11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AG11" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AH11" t="s" s="19">
+      <c r="L11" t="s" s="18">
         <v>116</v>
       </c>
+      <c r="M11" t="s" s="18">
+        <v>117</v>
+      </c>
+      <c r="N11" t="s" s="18">
+        <v>118</v>
+      </c>
+      <c r="O11" t="s" s="18">
+        <v>119</v>
+      </c>
+      <c r="P11" t="s" s="18">
+        <v>120</v>
+      </c>
+      <c r="Q11" t="s" s="18">
+        <v>121</v>
+      </c>
+      <c r="R11" t="s" s="18">
+        <v>122</v>
+      </c>
+      <c r="S11" t="s" s="18">
+        <v>123</v>
+      </c>
+      <c r="T11" t="s" s="18">
+        <v>124</v>
+      </c>
+      <c r="U11" t="s" s="18">
+        <v>125</v>
+      </c>
+      <c r="V11" t="s" s="18">
+        <v>126</v>
+      </c>
+      <c r="W11" t="s" s="18">
+        <v>127</v>
+      </c>
+      <c r="X11" t="s" s="18">
+        <v>128</v>
+      </c>
+      <c r="Y11" t="s" s="18">
+        <v>129</v>
+      </c>
+      <c r="Z11" t="s" s="18">
+        <v>130</v>
+      </c>
+      <c r="AA11" t="s" s="18">
+        <v>131</v>
+      </c>
+      <c r="AB11" t="s" s="18">
+        <v>132</v>
+      </c>
+      <c r="AC11" t="s" s="18">
+        <v>133</v>
+      </c>
+      <c r="AD11" t="s" s="18">
+        <v>134</v>
+      </c>
+      <c r="AE11" t="s" s="18">
+        <v>135</v>
+      </c>
+      <c r="AF11" t="s" s="18">
+        <v>136</v>
+      </c>
+      <c r="AG11" t="s" s="18">
+        <v>137</v>
+      </c>
+      <c r="AH11" t="s" s="18">
+        <v>138</v>
+      </c>
       <c r="AI11" t="s" s="19">
-        <v>117</v>
+        <v>139</v>
       </c>
     </row>
     <row r="12" ht="12.9" customHeight="1">
       <c r="A12" t="s" s="2">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="C12" t="s" s="19">
-        <v>113</v>
-      </c>
-      <c r="D12" t="s" s="19">
-        <v>114</v>
-      </c>
-      <c r="E12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AG12" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AH12" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI12" t="s" s="19">
-        <v>117</v>
+        <v>141</v>
+      </c>
+      <c r="C12" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D12" t="s" s="20">
+        <v>143</v>
+      </c>
+      <c r="E12" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="F12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG12" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH12" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI12" t="s" s="20">
+        <v>147</v>
       </c>
     </row>
     <row r="13" ht="12.9" customHeight="1">
       <c r="A13" t="s" s="2">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>120</v>
-      </c>
-      <c r="C13" t="s" s="19">
-        <v>113</v>
-      </c>
-      <c r="D13" t="s" s="19">
-        <v>121</v>
-      </c>
-      <c r="E13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AG13" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AH13" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI13" t="s" s="19">
-        <v>122</v>
+        <v>141</v>
+      </c>
+      <c r="C13" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D13" t="s" s="20">
+        <v>143</v>
+      </c>
+      <c r="E13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F13" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="G13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG13" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH13" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI13" t="s" s="20">
+        <v>147</v>
       </c>
     </row>
     <row r="14" ht="12.9" customHeight="1">
       <c r="A14" t="s" s="2">
-        <v>123</v>
+        <v>149</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>124</v>
-      </c>
-      <c r="C14" t="s" s="19">
-        <v>113</v>
-      </c>
-      <c r="D14" t="s" s="19">
-        <v>125</v>
-      </c>
-      <c r="E14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AG14" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AH14" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI14" t="s" s="19">
-        <v>126</v>
+        <v>141</v>
+      </c>
+      <c r="C14" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D14" t="s" s="20">
+        <v>143</v>
+      </c>
+      <c r="E14" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="F14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G14" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="H14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG14" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH14" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI14" t="s" s="20">
+        <v>147</v>
       </c>
     </row>
     <row r="15" ht="12.9" customHeight="1">
       <c r="A15" t="s" s="2">
-        <v>127</v>
+        <v>150</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>128</v>
-      </c>
-      <c r="C15" t="s" s="19">
-        <v>121</v>
-      </c>
-      <c r="D15" t="s" s="19">
-        <v>114</v>
-      </c>
-      <c r="E15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF15" t="s" s="19">
-        <v>129</v>
-      </c>
-      <c r="AG15" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AH15" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI15" t="s" s="19">
-        <v>117</v>
+        <v>151</v>
+      </c>
+      <c r="C15" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D15" t="s" s="20">
+        <v>152</v>
+      </c>
+      <c r="E15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG15" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH15" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI15" t="s" s="20">
+        <v>153</v>
       </c>
     </row>
     <row r="16" ht="12.9" customHeight="1">
       <c r="A16" t="s" s="2">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="C16" t="s" s="19">
-        <v>113</v>
-      </c>
-      <c r="D16" t="s" s="19">
-        <v>132</v>
-      </c>
-      <c r="E16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF16" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AG16" t="s" s="19">
-        <v>129</v>
-      </c>
-      <c r="AH16" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI16" t="s" s="19">
-        <v>133</v>
+        <v>155</v>
+      </c>
+      <c r="C16" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D16" t="s" s="20">
+        <v>156</v>
+      </c>
+      <c r="E16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG16" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH16" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI16" t="s" s="20">
+        <v>157</v>
       </c>
     </row>
     <row r="17" ht="12.9" customHeight="1">
       <c r="A17" t="s" s="2">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="C17" t="s" s="19">
-        <v>113</v>
-      </c>
-      <c r="D17" t="s" s="19">
-        <v>132</v>
-      </c>
-      <c r="E17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AF17" t="s" s="19">
-        <v>129</v>
-      </c>
-      <c r="AG17" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AH17" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI17" t="s" s="19">
-        <v>133</v>
+        <v>159</v>
+      </c>
+      <c r="C17" t="s" s="20">
+        <v>152</v>
+      </c>
+      <c r="D17" t="s" s="20">
+        <v>143</v>
+      </c>
+      <c r="E17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF17" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="AG17" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH17" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI17" t="s" s="20">
+        <v>147</v>
       </c>
     </row>
     <row r="18" ht="12.9" customHeight="1">
       <c r="A18" t="s" s="2">
-        <v>135</v>
+        <v>160</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>131</v>
-      </c>
-      <c r="C18" t="s" s="19">
-        <v>113</v>
-      </c>
-      <c r="D18" t="s" s="19">
-        <v>132</v>
-      </c>
-      <c r="E18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="F18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="G18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="H18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="I18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="J18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="K18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="L18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="M18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="N18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="O18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="P18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Q18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="R18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="S18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="T18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="U18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="V18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="W18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="X18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Y18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="Z18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AA18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AB18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AC18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AD18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AE18" t="s" s="19">
-        <v>129</v>
-      </c>
-      <c r="AF18" t="s" s="19">
-        <v>115</v>
-      </c>
-      <c r="AG18" t="s" s="19">
-        <v>129</v>
-      </c>
-      <c r="AH18" t="s" s="19">
-        <v>116</v>
-      </c>
-      <c r="AI18" t="s" s="19">
-        <v>133</v>
+        <v>161</v>
+      </c>
+      <c r="C18" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D18" t="s" s="20">
+        <v>162</v>
+      </c>
+      <c r="E18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF18" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG18" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="AH18" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI18" t="s" s="20">
+        <v>163</v>
       </c>
     </row>
     <row r="19" ht="12.9" customHeight="1">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="19"/>
-      <c r="P19" s="19"/>
-      <c r="Q19" s="19"/>
-      <c r="R19" s="19"/>
-      <c r="S19" s="19"/>
-      <c r="T19" s="19"/>
-      <c r="U19" s="19"/>
-      <c r="V19" s="19"/>
-      <c r="W19" s="19"/>
-      <c r="X19" s="19"/>
-      <c r="Y19" s="19"/>
-      <c r="Z19" s="19"/>
-      <c r="AA19" s="19"/>
-      <c r="AB19" s="19"/>
-      <c r="AC19" s="19"/>
-      <c r="AD19" s="19"/>
-      <c r="AE19" s="19"/>
-      <c r="AF19" s="19"/>
-      <c r="AG19" s="19"/>
-      <c r="AH19" s="19"/>
-      <c r="AI19" s="19"/>
+      <c r="A19" t="s" s="2">
+        <v>164</v>
+      </c>
+      <c r="B19" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="C19" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D19" t="s" s="20">
+        <v>162</v>
+      </c>
+      <c r="E19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AF19" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="AG19" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AH19" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI19" t="s" s="20">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="20" ht="12.9" customHeight="1">
+      <c r="A20" t="s" s="2">
+        <v>165</v>
+      </c>
+      <c r="B20" t="s" s="2">
+        <v>161</v>
+      </c>
+      <c r="C20" t="s" s="20">
+        <v>142</v>
+      </c>
+      <c r="D20" t="s" s="20">
+        <v>162</v>
+      </c>
+      <c r="E20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="F20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="G20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="H20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="I20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="J20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="K20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="L20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="M20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="N20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="O20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="P20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Q20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="R20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="S20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="T20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="U20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="V20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="W20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="X20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Y20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="Z20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AA20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AB20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AC20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AD20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AE20" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="AF20" t="s" s="20">
+        <v>145</v>
+      </c>
+      <c r="AG20" t="s" s="20">
+        <v>144</v>
+      </c>
+      <c r="AH20" t="s" s="20">
+        <v>146</v>
+      </c>
+      <c r="AI20" t="s" s="20">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="21" ht="12.9" customHeight="1">
+      <c r="A21" s="2"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="20"/>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="20"/>
+      <c r="G21" s="20"/>
+      <c r="H21" s="20"/>
+      <c r="I21" s="20"/>
+      <c r="J21" s="20"/>
+      <c r="K21" s="20"/>
+      <c r="L21" s="20"/>
+      <c r="M21" s="20"/>
+      <c r="N21" s="20"/>
+      <c r="O21" s="20"/>
+      <c r="P21" s="20"/>
+      <c r="Q21" s="20"/>
+      <c r="R21" s="20"/>
+      <c r="S21" s="20"/>
+      <c r="T21" s="20"/>
+      <c r="U21" s="20"/>
+      <c r="V21" s="20"/>
+      <c r="W21" s="20"/>
+      <c r="X21" s="20"/>
+      <c r="Y21" s="20"/>
+      <c r="Z21" s="20"/>
+      <c r="AA21" s="20"/>
+      <c r="AB21" s="20"/>
+      <c r="AC21" s="20"/>
+      <c r="AD21" s="20"/>
+      <c r="AE21" s="20"/>
+      <c r="AF21" s="20"/>
+      <c r="AG21" s="20"/>
+      <c r="AH21" s="20"/>
+      <c r="AI21" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>